<commit_message>
Updated weekly report 04-30
</commit_message>
<xml_diff>
--- a/ECE554-weekly-report.xlsx
+++ b/ECE554-weekly-report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t>Name</t>
   </si>
@@ -34,33 +34,58 @@
     <t>Week 6</t>
   </si>
   <si>
+    <t>Week 7</t>
+  </si>
+  <si>
+    <t>Week 8</t>
+  </si>
+  <si>
+    <t>Week 9</t>
+  </si>
+  <si>
     <t>Anirudh Kompella</t>
   </si>
   <si>
-    <t>- Created Project Proposal document
+    <t>- Created project proposal document outlining system design and objectives
 - Researched Catapult C conversion from C++ to Verilog</t>
   </si>
   <si>
     <t>-Created IO Devices Presentation
 - Implemented calibration mode (SW[8]) with center sampling + RGB capture
--Wrote Verilog Tests for top Layer</t>
-  </si>
-  <si>
-    <t>-Designed and implemented the snake block module
--Developed core snake game logic
+-Wrote Verilog Tests for top Layer + Developed microarchitecture for color capture logic</t>
+  </si>
+  <si>
+    <t>-Designed and implemented the snake block module with core logic 
+-Implemented two-flip-flop CDC synchroniser for all camera-to-VGA domain signals (top level)
 -Added rendering system for snake game visuals</t>
   </si>
   <si>
-    <t>- Created Snake Game test file
+    <t>- Created comprehensive snake Game test file
 - Ran Snake Game logc into vidis HDL and generated Verilog files for top level</t>
   </si>
   <si>
     <t>-Developed capstone website showcasing team and project
--Maintained site with updates, progress, and resources</t>
-  </si>
-  <si>
-    <t>-Created testbenches for key modules
--Debugged Key modules and test benches</t>
+-Maintained site with updates, progress, and resources
+-Engineered brightness threshold to reject near-black false-positive matches (with Chance)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-Created comprehensive testbenches for key modules validating correct hardware behaviour
+- Implemented frame divider to control snake movement speed precisely  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Implemented a 20x15 grid canvas using single-bit FPGA registers in draw game
+- Built hand detection integration using centroid coordinates from color_detect                                             
+- Designed three-priority pixel renderer for cursor, painted cells, background </t>
+  </si>
+  <si>
+    <t>- Built catch game with real-time hand tracking
+- Designed dynamic difficulty scaling using score thresholds                                             
+- Implemented VGA pixel renderer with custom glyphs</t>
+  </si>
+  <si>
+    <t>- Updated catch game with pseudo-random object spawning via LFSR logic
+- Rendered scaled bitmap glyphs for live scoreboard and win banner for Pong game                                            
+- Written comprehensive testbench for all the games</t>
   </si>
   <si>
     <t>Chance Howarth</t>
@@ -76,7 +101,8 @@
 -Added LED indicators and refined exposure controls</t>
   </si>
   <si>
-    <t>-Developed visual overlay (tracking box + center marker)
+    <t>-Routed I2C interface to configure D5M camera sensor registers over SCLK
+-Developed visual overlay (tracking box + center marker)
 -Added real-time debugging visuals (live RGB, tracking feedback)</t>
   </si>
   <si>
@@ -85,8 +111,27 @@
  -Integrated zoom mode and control refinements</t>
   </si>
   <si>
-    <t>-Developed buffer to improve camera tracking
--Debugged Key modules and test benches</t>
+    <t>-Developed bounding box output to localise the detected colour region
+-Engineered brightness threshold to reject near-black false-positive matches (with Anirudh)
+-Designed tolerance scaling system that adapts to varying lighting conditions</t>
+  </si>
+  <si>
+    <t>-Developed frame buffer to stabilise and improve real-time camera tracking
+-Debugged key hardware modules and testbenches to ensure correct functionality</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Fixed inverted direction tracking on draw game                                                   
+  - Synthesized design using 300 flip-flops sharing the 25 MHz VGA clock</t>
+  </si>
+  <si>
+    <t>- Built two-player hand-tracked Pong using colour detection and VGA output
+- Implemented signed velocity ball physics with per-hit speed acceleration                                             
+- Rendered scaled bitmap glyphs for live scoreboard and win banner</t>
+  </si>
+  <si>
+    <t>- Implemented Bresenham line algorithm for smooth strokes in draw game
+- Created pencil sprite with pen-state colour feedback in draw game                                            
+- Refined 2 color tracking for the Pong game.</t>
   </si>
   <si>
     <t>Amer Salem</t>
@@ -114,22 +159,46 @@
 -Looked into pixel warping issue</t>
   </si>
   <si>
-    <t>-Updated the Snake game to allow right to left tracking</t>
+    <t xml:space="preserve">-Updated the Snake game to allow right to left tracking
+- Added game states and a start screen
+</t>
+  </si>
+  <si>
+    <t>- Added Score Tracking into FSM and UI Component to snake Game
+- Implemented head-relative dead zone to prevent unintended direction changes                                             
+- Created deterministic food sequence cycling through ten pre-set grid positions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Instantiated separate renderer module keeping game logic cleanly decoupled
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Created a poster with clear sections covering algorithms, rendering, and peripherals
+</t>
   </si>
   <si>
     <t>Munasib Ilham</t>
   </si>
   <si>
-    <t xml:space="preserve">- Researched Verilog best practices and </t>
-  </si>
-  <si>
-    <t>-Created micro architecture Diagram and Slides</t>
-  </si>
-  <si>
-    <t>-Created Architecture Block Diagram and slides</t>
-  </si>
-  <si>
-    <t>- Optimized Snake game to Compile faser</t>
+    <t>-Looked into hardware architecture design for our project</t>
+  </si>
+  <si>
+    <t>-Built initial top level code for FPGA interface
+-Developed microarchitecture for color capture logic</t>
+  </si>
+  <si>
+    <t>-Created micro architecture Diagram and Slides
+-Developed graphics rendering pipeline for the game</t>
+  </si>
+  <si>
+    <t>- Optimized Snake game to Compile faster
+- Looking at ways to fix synchronization issue between VGA clock speed and verilog module clock speed</t>
+  </si>
+  <si>
+    <t>-Added Game Over UI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Writing the final report </t>
   </si>
 </sst>
 </file>
@@ -258,8 +327,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A1:G1" displayName="Table1" name="Table1" id="1">
-  <tableColumns count="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A1:J1" displayName="Table1" name="Table1" id="1">
+  <tableColumns count="10">
     <tableColumn name="Column1" id="1"/>
     <tableColumn name="Column2" id="2"/>
     <tableColumn name="Column3" id="3"/>
@@ -267,6 +336,9 @@
     <tableColumn name="Column5" id="5"/>
     <tableColumn name="Column6" id="6"/>
     <tableColumn name="Column7" id="7"/>
+    <tableColumn name="Column8" id="8"/>
+    <tableColumn name="Column9" id="9"/>
+    <tableColumn name="Column10" id="10"/>
   </tableColumns>
   <tableStyleInfo name="Sheet1-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
   <extLst>
@@ -481,10 +553,13 @@
     <col customWidth="1" min="1" max="1" width="17.5"/>
     <col customWidth="1" min="2" max="2" width="69.0"/>
     <col customWidth="1" min="3" max="3" width="58.13"/>
-    <col customWidth="1" min="4" max="4" width="52.25"/>
+    <col customWidth="1" min="4" max="4" width="71.25"/>
     <col customWidth="1" min="5" max="5" width="59.13"/>
-    <col customWidth="1" min="6" max="6" width="63.25"/>
-    <col customWidth="1" min="7" max="7" width="22.13"/>
+    <col customWidth="1" min="6" max="6" width="75.25"/>
+    <col customWidth="1" min="7" max="7" width="78.13"/>
+    <col customWidth="1" min="8" max="8" width="83.38"/>
+    <col customWidth="1" min="9" max="9" width="61.0"/>
+    <col customWidth="1" min="10" max="10" width="63.0"/>
   </cols>
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
@@ -509,89 +584,142 @@
       <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>13</v>
+        <v>16</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>18</v>
+        <v>24</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>19</v>
+        <v>26</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>26</v>
+        <v>36</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>28</v>
+        <v>41</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>42</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>31</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="H7" s="4"/>
+      <c r="J7" s="4"/>
+    </row>
+    <row r="8">
+      <c r="H8" s="4"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>